<commit_message>
Connect scraper to Flask deployment
</commit_message>
<xml_diff>
--- a/naukri_jobs.xlsx
+++ b/naukri_jobs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1335,10 +1335,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>240826007480</t>
-        </is>
+      <c r="A24" t="n">
+        <v>240826007480</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1377,10 +1375,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>170626036185</t>
-        </is>
+      <c r="A25" t="n">
+        <v>170626036185</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1419,10 +1415,8 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>050925009110</t>
-        </is>
+      <c r="A26" t="n">
+        <v>50925009110</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1461,10 +1455,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>300826004292</t>
-        </is>
+      <c r="A27" t="n">
+        <v>300826004292</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1503,10 +1495,8 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>150926017345</t>
-        </is>
+      <c r="A28" t="n">
+        <v>150926017345</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1545,10 +1535,8 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>250926500051</t>
-        </is>
+      <c r="A29" t="n">
+        <v>250926500051</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1587,10 +1575,8 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>250926036504</t>
-        </is>
+      <c r="A30" t="n">
+        <v>250926036504</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1629,10 +1615,8 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>250926036398</t>
-        </is>
+      <c r="A31" t="n">
+        <v>250926036398</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1671,10 +1655,8 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>250926034242</t>
-        </is>
+      <c r="A32" t="n">
+        <v>250926034242</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1713,10 +1695,8 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>250926036403</t>
-        </is>
+      <c r="A33" t="n">
+        <v>250926036403</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1755,10 +1735,8 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>250926034317</t>
-        </is>
+      <c r="A34" t="n">
+        <v>250926034317</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1797,10 +1775,8 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>210926001708</t>
-        </is>
+      <c r="A35" t="n">
+        <v>210926001708</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1839,10 +1815,8 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>250926018972</t>
-        </is>
+      <c r="A36" t="n">
+        <v>250926018972</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1881,10 +1855,8 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>250926037488</t>
-        </is>
+      <c r="A37" t="n">
+        <v>250926037488</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1923,10 +1895,8 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>210926026375</t>
-        </is>
+      <c r="A38" t="n">
+        <v>210926026375</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1965,10 +1935,8 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>260926008983</t>
-        </is>
+      <c r="A39" t="n">
+        <v>260926008983</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -2007,10 +1975,8 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>240926042072</t>
-        </is>
+      <c r="A40" t="n">
+        <v>240926042072</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -2049,10 +2015,8 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>250926037677</t>
-        </is>
+      <c r="A41" t="n">
+        <v>250926037677</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -2087,6 +2051,90 @@
       <c r="H41" t="inlineStr">
         <is>
           <t>https://www.naukri.com/job-listings-python-developer-shree-trishakti-group-hyderabad-pune-chennai-7-to-12-years-250926037677</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>250926035861</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Python Developer (5 To 8 Years)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Infosys</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Hybrid - Noida, Hyderabad, Bengaluru</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>5-8 Yrs</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>DjangoPython DeveloperPythonPython DevelopmentFlaskDevelopment</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2 days ago</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-python-developer-5-to-8-years-infosys-noida-hyderabad-bengaluru-5-to-8-years-250926035861</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>230926020364</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Python Developer</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Naukri E-hire</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Pune, Chennai, Bengaluru</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>6-9 Yrs</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>PysparkPythonDjango FrameworkPython DevelopmentSenior Systems EngineerSeniorSystemFramework</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>4 days ago</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>https://www.naukri.com/job-listings-python-developer-naukri-e-hire-pune-chennai-bengaluru-6-to-9-years-230926020364</t>
         </is>
       </c>
     </row>

</xml_diff>